<commit_message>
Add nine Russian thematic hashtags per SKU and update audit
</commit_message>
<xml_diff>
--- a/ozon/phase1/20261028-0000/ozon_phase1_audit.xlsx
+++ b/ozon/phase1/20261028-0000/ozon_phase1_audit.xlsx
@@ -14,6 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="待确认事项" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="字段对应及空值" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="检查与未完成" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="九个主题标签" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'使用说明'!$A$1:$B$13</definedName>
@@ -23,6 +24,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'待确认事项'!$A$1:$C$36</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'字段对应及空值'!$A$1:$B$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'检查与未完成'!$A$1:$C$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'九个主题标签'!$A$1:$G$44</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -69,10 +71,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -551,7 +556,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>模板禁止品牌、参数、产品名称；无明确风格主题支持，Y留空，未编造标签。</t>
+          <t>按用户追加要求，每SKU填写9个俄文主题标签；依商品用途分装饰/维修两组。未取得Ozon搜索量、销量或标签热榜，不声称为已验证爆款标签。</t>
         </is>
       </c>
     </row>
@@ -7175,7 +7180,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>无符合模板且有资料支持的主题风格标签，Y留空。</t>
+          <t>按用户追加要求，每SKU填写9个俄文主题标签；依商品用途分装饰/维修两组。未取得Ozon搜索量、销量或标签热榜，不声称为已验证爆款标签。</t>
         </is>
       </c>
     </row>
@@ -7797,7 +7802,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>无有支持且符合模板的主题标签留空。</t>
+          <t>按用户追加要求，每SKU填写9个俄文主题标签；依商品用途分装饰/维修两组。未取得Ozon搜索量、销量或标签热榜，不声称为已验证爆款标签。</t>
         </is>
       </c>
     </row>
@@ -7825,7 +7830,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -8088,8 +8093,1505 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>9个主题标签</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>通过（格式及数量）</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>43个SKU各9个；俄文、#开头、空格分隔、每个不超30字符、单行不重复；无品牌/产品名称/参数；Ozon爆款热度未验证。</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:C15"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G44"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="90" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>原款号</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>新款号</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>模板行</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>主题分组</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>标签数量</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>俄文标签</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>Ozon热度验证状态</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>2018YF078_5</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH078_5</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>维修更新主题</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>#авторемонт #ремонтавтомобиля #восстановлениеавто #обновлениеавто #автопроект #гаражныйпроект #гараж #автолюбитель #автотема</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>未验证；无Ozon实时搜索量、销量及标签热榜数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>2018YF078_6</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH078_6</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>维修更新主题</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>#авторемонт #ремонтавтомобиля #восстановлениеавто #обновлениеавто #автопроект #гаражныйпроект #гараж #автолюбитель #автотема</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>未验证；无Ozon实时搜索量、销量及标签热榜数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>2018YF078_4</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH078_4</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>维修更新主题</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>#авторемонт #ремонтавтомобиля #восстановлениеавто #обновлениеавто #автопроект #гаражныйпроект #гараж #автолюбитель #автотема</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>未验证；无Ozon实时搜索量、销量及标签热榜数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>2018YF078_3</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH078_3</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>维修更新主题</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>#авторемонт #ремонтавтомобиля #восстановлениеавто #обновлениеавто #автопроект #гаражныйпроект #гараж #автолюбитель #автотема</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>未验证；无Ozon实时搜索量、销量及标签热榜数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>2018YF078_2</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH078_2</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>维修更新主题</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>#авторемонт #ремонтавтомобиля #восстановлениеавто #обновлениеавто #автопроект #гаражныйпроект #гараж #автолюбитель #автотема</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>未验证；无Ozon实时搜索量、销量及标签热榜数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>2018YF078_1</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH078_1</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>维修更新主题</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>#авторемонт #ремонтавтомобиля #восстановлениеавто #обновлениеавто #автопроект #гаражныйпроект #гараж #автолюбитель #автотема</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>未验证；无Ozon实时搜索量、销量及标签热榜数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>2018YF077_4</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH077_4</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>维修更新主题</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>#авторемонт #ремонтавтомобиля #восстановлениеавто #обновлениеавто #автопроект #гаражныйпроект #гараж #автолюбитель #автотема</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>未验证；无Ozon实时搜索量、销量及标签热榜数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>2018YF077_3</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH077_3</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>维修更新主题</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>#авторемонт #ремонтавтомобиля #восстановлениеавто #обновлениеавто #автопроект #гаражныйпроект #гараж #автолюбитель #автотема</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>未验证；无Ozon实时搜索量、销量及标签热榜数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>2018YF077_2</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH077_2</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>维修更新主题</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>#авторемонт #ремонтавтомобиля #восстановлениеавто #обновлениеавто #автопроект #гаражныйпроект #гараж #автолюбитель #автотема</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>未验证；无Ozon实时搜索量、销量及标签热榜数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>2018YF077_1</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH077_1</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>维修更新主题</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>#авторемонт #ремонтавтомобиля #восстановлениеавто #обновлениеавто #автопроект #гаражныйпроект #гараж #автолюбитель #автотема</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>未验证；无Ozon实时搜索量、销量及标签热榜数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>2018YF076_4</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH076_4</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>维修更新主题</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>#авторемонт #ремонтавтомобиля #восстановлениеавто #обновлениеавто #автопроект #гаражныйпроект #гараж #автолюбитель #автотема</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>未验证；无Ozon实时搜索量、销量及标签热榜数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>2018YF075</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH075</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>维修更新主题</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>#авторемонт #ремонтавтомобиля #восстановлениеавто #обновлениеавто #автопроект #гаражныйпроект #гараж #автолюбитель #автотема</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>未验证；无Ozon实时搜索量、销量及标签热榜数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>2018YF074</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH074</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>维修更新主题</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>#авторемонт #ремонтавтомобиля #восстановлениеавто #обновлениеавто #автопроект #гаражныйпроект #гараж #автолюбитель #автотема</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>未验证；无Ozon实时搜索量、销量及标签热榜数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>2018YF073</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH073</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>外观装饰主题</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>#автостиль #автоэстетика #автодизайн #стильавтомобиля #обновлениеавто #автопроект #автолюбитель #автотема #тюнинг</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>未验证；无Ozon实时搜索量、销量及标签热榜数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>2018YF072</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH072</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>外观装饰主题</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>#автостиль #автоэстетика #автодизайн #стильавтомобиля #обновлениеавто #автопроект #автолюбитель #автотема #тюнинг</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>未验证；无Ozon实时搜索量、销量及标签热榜数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>2018YF071</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH071</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>外观装饰主题</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>#автостиль #автоэстетика #автодизайн #стильавтомобиля #обновлениеавто #автопроект #автолюбитель #автотема #тюнинг</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>未验证；无Ozon实时搜索量、销量及标签热榜数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>2018YF070</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH070</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>外观装饰主题</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>#автостиль #автоэстетика #автодизайн #стильавтомобиля #обновлениеавто #автопроект #автолюбитель #автотема #тюнинг</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>未验证；无Ozon实时搜索量、销量及标签热榜数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>2018YF069</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH069</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>外观装饰主题</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>#автостиль #автоэстетика #автодизайн #стильавтомобиля #обновлениеавто #автопроект #автолюбитель #автотема #тюнинг</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>未验证；无Ozon实时搜索量、销量及标签热榜数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>2018YF068</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH068</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>外观装饰主题</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>#автостиль #автоэстетика #автодизайн #стильавтомобиля #обновлениеавто #автопроект #автолюбитель #автотема #тюнинг</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>未验证；无Ozon实时搜索量、销量及标签热榜数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>2018YF067</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH067</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>外观装饰主题</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>#автостиль #автоэстетика #автодизайн #стильавтомобиля #обновлениеавто #автопроект #автолюбитель #автотема #тюнинг</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>未验证；无Ozon实时搜索量、销量及标签热榜数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>2018YF065</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH065</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>外观装饰主题</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>#автостиль #автоэстетика #автодизайн #стильавтомобиля #обновлениеавто #автопроект #автолюбитель #автотема #тюнинг</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>未验证；无Ozon实时搜索量、销量及标签热榜数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>2018YF064</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH064</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>外观装饰主题</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>#автостиль #автоэстетика #автодизайн #стильавтомобиля #обновлениеавто #автопроект #автолюбитель #автотема #тюнинг</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>未验证；无Ozon实时搜索量、销量及标签热榜数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>2018YF063</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH063</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>外观装饰主题</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>#автостиль #автоэстетика #автодизайн #стильавтомобиля #обновлениеавто #автопроект #автолюбитель #автотема #тюнинг</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>未验证；无Ozon实时搜索量、销量及标签热榜数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>2018YF062</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH062</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>外观装饰主题</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>#автостиль #автоэстетика #автодизайн #стильавтомобиля #обновлениеавто #автопроект #автолюбитель #автотема #тюнинг</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>未验证；无Ozon实时搜索量、销量及标签热榜数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>2018YF061</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH061</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>外观装饰主题</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>#автостиль #автоэстетика #автодизайн #стильавтомобиля #обновлениеавто #автопроект #автолюбитель #автотема #тюнинг</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>未验证；无Ozon实时搜索量、销量及标签热榜数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>2018YF060</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH060</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>外观装饰主题</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>#автостиль #автоэстетика #автодизайн #стильавтомобиля #обновлениеавто #автопроект #автолюбитель #автотема #тюнинг</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>未验证；无Ozon实时搜索量、销量及标签热榜数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>2018YF059</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH059</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>外观装饰主题</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>#автостиль #автоэстетика #автодизайн #стильавтомобиля #обновлениеавто #автопроект #автолюбитель #автотема #тюнинг</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>未验证；无Ozon实时搜索量、销量及标签热榜数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>2018YF058</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH058</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>外观装饰主题</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>#автостиль #автоэстетика #автодизайн #стильавтомобиля #обновлениеавто #автопроект #автолюбитель #автотема #тюнинг</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>未验证；无Ozon实时搜索量、销量及标签热榜数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>2018YF057</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH057</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>外观装饰主题</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>#автостиль #автоэстетика #автодизайн #стильавтомобиля #обновлениеавто #автопроект #автолюбитель #автотема #тюнинг</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>未验证；无Ozon实时搜索量、销量及标签热榜数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>2018YF056</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH056</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>外观装饰主题</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>#автостиль #автоэстетика #автодизайн #стильавтомобиля #обновлениеавто #автопроект #автолюбитель #автотема #тюнинг</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>未验证；无Ozon实时搜索量、销量及标签热榜数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>2018YF055</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH055</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>外观装饰主题</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>#автостиль #автоэстетика #автодизайн #стильавтомобиля #обновлениеавто #автопроект #автолюбитель #автотема #тюнинг</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>未验证；无Ozon实时搜索量、销量及标签热榜数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>2018YF054</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH054</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>外观装饰主题</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>#автостиль #автоэстетика #автодизайн #стильавтомобиля #обновлениеавто #автопроект #автолюбитель #автотема #тюнинг</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>未验证；无Ozon实时搜索量、销量及标签热榜数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>2018YF053</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH053</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>外观装饰主题</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>#автостиль #автоэстетика #автодизайн #стильавтомобиля #обновлениеавто #автопроект #автолюбитель #автотема #тюнинг</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>未验证；无Ozon实时搜索量、销量及标签热榜数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>2018YF052</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH052</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>维修更新主题</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>#авторемонт #ремонтавтомобиля #восстановлениеавто #обновлениеавто #автопроект #гаражныйпроект #гараж #автолюбитель #автотема</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>未验证；无Ozon实时搜索量、销量及标签热榜数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>2018YF051PT</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH051PT</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>维修更新主题</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>#авторемонт #ремонтавтомобиля #восстановлениеавто #обновлениеавто #автопроект #гаражныйпроект #гараж #автолюбитель #автотема</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>未验证；无Ozon实时搜索量、销量及标签热榜数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>2018YF051</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH051</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>维修更新主题</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>#авторемонт #ремонтавтомобиля #восстановлениеавто #обновлениеавто #автопроект #гаражныйпроект #гараж #автолюбитель #автотема</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>未验证；无Ozon实时搜索量、销量及标签热榜数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>2018YF050</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH050</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>维修更新主题</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>#авторемонт #ремонтавтомобиля #восстановлениеавто #обновлениеавто #автопроект #гаражныйпроект #гараж #автолюбитель #автотема</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>未验证；无Ozon实时搜索量、销量及标签热榜数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>2018YF049PT</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH049PT</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>维修更新主题</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>#авторемонт #ремонтавтомобиля #восстановлениеавто #обновлениеавто #автопроект #гаражныйпроект #гараж #автолюбитель #автотема</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>未验证；无Ozon实时搜索量、销量及标签热榜数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>2018YF048</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH048</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>维修更新主题</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>#авторемонт #ремонтавтомобиля #восстановлениеавто #обновлениеавто #автопроект #гаражныйпроект #гараж #автолюбитель #автотема</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>未验证；无Ozon实时搜索量、销量及标签热榜数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>2018YF047</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH047</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>维修更新主题</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>#авторемонт #ремонтавтомобиля #восстановлениеавто #обновлениеавто #автопроект #гаражныйпроект #гараж #автолюбитель #автотема</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>未验证；无Ozon实时搜索量、销量及标签热榜数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>2018YF046PT</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH046PT</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>维修更新主题</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>#авторемонт #ремонтавтомобиля #восстановлениеавто #обновлениеавто #автопроект #гаражныйпроект #гараж #автолюбитель #автотема</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>未验证；无Ozon实时搜索量、销量及标签热榜数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>2018YF045</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH045</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>维修更新主题</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>#авторемонт #ремонтавтомобиля #восстановлениеавто #обновлениеавто #автопроект #гаражныйпроект #гараж #автолюбитель #автотема</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>未验证；无Ozon实时搜索量、销量及标签热榜数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>2018YF044QH</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>3018WYH044QH</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="n">
+        <v>47</v>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>维修更新主题</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>#авторемонт #ремонтавтомобиля #восстановлениеавто #обновлениеавто #автопроект #гаражныйпроект #гараж #автолюбитель #автотема</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>未验证；无Ozon实时搜索量、销量及标签热榜数据</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G44"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>